<commit_message>
Actualización SISTEMA PRO SEP2026
</commit_message>
<xml_diff>
--- a/BASE_RECORRIDOS_PRO_JCA.xlsx
+++ b/BASE_RECORRIDOS_PRO_JCA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\INTERVENTORIA VELNEC\Recorridos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9A81BD-C59B-405A-9957-E01AC8A41196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD2C1E5-DC97-41D2-9A03-66630DB74FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GRAFICAS" sheetId="7" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4577" uniqueCount="1671">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4711" uniqueCount="1727">
   <si>
     <t>ID</t>
   </si>
@@ -5062,7 +5062,175 @@
     <t>6.243433, -75.602993</t>
   </si>
   <si>
-    <t>retubieron el vehiculo donde estaba laborando en el corregimineto de Santa Elena</t>
+    <t>retuvieron el vehículo donde estaba laborando en el corregimiento de Santa Elena</t>
+  </si>
+  <si>
+    <t>d7b664ef81ad9651</t>
+  </si>
+  <si>
+    <t>18_09_2026_DV_Noct1.gpx</t>
+  </si>
+  <si>
+    <t>d7b664ef81ad9651554f4d4fa4321cd936eac554b8e90b2d1b9a7efec9642fb0</t>
+  </si>
+  <si>
+    <t>18/09/2026 18:14:24</t>
+  </si>
+  <si>
+    <t>18/09/2026 23:07:55</t>
+  </si>
+  <si>
+    <t>Inicio GPS dentro de la tolerancia del horario programado.; Fin GPS anticipado: 00:52:05 antes de las 00:00.; 1 hueco(s) GPS &gt;= 10 min.</t>
+  </si>
+  <si>
+    <t>6.270135, -75.601358</t>
+  </si>
+  <si>
+    <t>6.246358, -75.604612</t>
+  </si>
+  <si>
+    <t>0b3b3e04436c9877</t>
+  </si>
+  <si>
+    <t>18_09_2026_DV_Noct2.gpx</t>
+  </si>
+  <si>
+    <t>0b3b3e04436c9877c98cc7e76170acac75d69b6bfb77bc702a6e8b91134c7379</t>
+  </si>
+  <si>
+    <t>18/09/2026 22:19:50</t>
+  </si>
+  <si>
+    <t>19/09/2026 00:13:49</t>
+  </si>
+  <si>
+    <t>Inicio GPS tardío: 04:19:51 después de las 18:00.; Fin GPS dentro de la tolerancia del horario programado.; 1 hueco(s) GPS &gt;= 10 min.</t>
+  </si>
+  <si>
+    <t>6.251355, -75.607428</t>
+  </si>
+  <si>
+    <t>6.272566, -75.602164</t>
+  </si>
+  <si>
+    <t>411c6fb03be049a0</t>
+  </si>
+  <si>
+    <t>18_09_2026_IQ_Noct.gpx</t>
+  </si>
+  <si>
+    <t>411c6fb03be049a075a3b26e6982874b7088874c41de9683287188622862b445</t>
+  </si>
+  <si>
+    <t>18/09/2026 18:02:40</t>
+  </si>
+  <si>
+    <t>18/09/2026 23:44:35</t>
+  </si>
+  <si>
+    <t>Inicio GPS dentro de la tolerancia del horario programado.; Fin GPS anticipado: 00:15:25 antes de las 00:00.; 3 hueco(s) GPS &gt;= 10 min.</t>
+  </si>
+  <si>
+    <t>6.271953, -75.540673</t>
+  </si>
+  <si>
+    <t>6.264430, -75.570660</t>
+  </si>
+  <si>
+    <t>1c33940de6d83ac0</t>
+  </si>
+  <si>
+    <t>18_09_2026_JHP_Noct.gpx</t>
+  </si>
+  <si>
+    <t>1c33940de6d83ac0ea53dec915860f2c48d3fa189da38e1c9f34d7786ab4c7ba</t>
+  </si>
+  <si>
+    <t>18/09/2026 17:31:58</t>
+  </si>
+  <si>
+    <t>19/09/2026 00:21:47</t>
+  </si>
+  <si>
+    <t>Inicio GPS anterior al horario: 00:28:02 antes de las 18:00.; Fin GPS posterior: 00:21:47 después de las 00:00.</t>
+  </si>
+  <si>
+    <t>6.290363, -75.546539</t>
+  </si>
+  <si>
+    <t>6.290377, -75.546586</t>
+  </si>
+  <si>
+    <t>1f282216ee6e37f2</t>
+  </si>
+  <si>
+    <t>18_09_2026_JP_Noct.gpx</t>
+  </si>
+  <si>
+    <t>1f282216ee6e37f2520889c4282cf35711e63dfc3ceb4eb4602373514907a767</t>
+  </si>
+  <si>
+    <t>18/09/2026 17:58:21</t>
+  </si>
+  <si>
+    <t>18/09/2026 23:59:00</t>
+  </si>
+  <si>
+    <t>6.252467, -75.551827</t>
+  </si>
+  <si>
+    <t>6.251812, -75.551810</t>
+  </si>
+  <si>
+    <t>4eaa6f0e3139ce9c</t>
+  </si>
+  <si>
+    <t>18_09_2026_LA_Noct.gpx</t>
+  </si>
+  <si>
+    <t>4eaa6f0e3139ce9c3a1da9d13c538d9ea5f60c113e3a1e72c2c5288d79d3016e</t>
+  </si>
+  <si>
+    <t>18/09/2026 17:27:27</t>
+  </si>
+  <si>
+    <t>19/09/2026 00:00:48</t>
+  </si>
+  <si>
+    <t>Inicio GPS anterior al horario: 00:32:33 antes de las 18:00.; Fin GPS dentro de la tolerancia del horario programado.; 2 hueco(s) GPS &gt;= 10 min.</t>
+  </si>
+  <si>
+    <t>6.268908, -75.598983</t>
+  </si>
+  <si>
+    <t>6.239752, -75.575770</t>
+  </si>
+  <si>
+    <t>3045fae0d268338d</t>
+  </si>
+  <si>
+    <t>19_09_2026_AR_Noct.gpx</t>
+  </si>
+  <si>
+    <t>3045fae0d268338d25d3cd23bdd9fd7b7ab66535277cf52b510b0f2255c64b2c</t>
+  </si>
+  <si>
+    <t>19/09/2026 18:23:21</t>
+  </si>
+  <si>
+    <t>20/09/2026 00:05:17</t>
+  </si>
+  <si>
+    <t>Inicio GPS tardío: 00:23:21 después de las 18:00.; Fin GPS dentro de la tolerancia del horario programado.; Sábado nocturno: verificar técnico asignado.</t>
+  </si>
+  <si>
+    <t>6.247751, -75.614997</t>
+  </si>
+  <si>
+    <t>6.247642, -75.614915</t>
+  </si>
+  <si>
+    <t>Este recorrido inicio temprano</t>
   </si>
 </sst>
 </file>
@@ -5374,6 +5542,14 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="26" formatCode="h:mm:ss"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="14"/>
+      </font>
+    </dxf>
+    <dxf>
       <font>
         <sz val="14"/>
       </font>
@@ -5429,11 +5605,9 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="26" formatCode="h:mm:ss"/>
-    </dxf>
-    <dxf>
       <font>
-        <sz val="14"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -5459,12 +5633,6 @@
     <dxf>
       <font>
         <sz val="14"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <name val="Arial"/>
-        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -39146,834 +39314,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D330A9A-54B8-43DD-8D11-CC5633B99CDA}" name="TablaDinámica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
-  <location ref="A6:E22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="32">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="18">
-        <item x="0"/>
-        <item x="1"/>
-        <item h="1" x="15"/>
-        <item x="2"/>
-        <item h="1" m="1" x="16"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="16">
-        <item x="1"/>
-        <item x="9"/>
-        <item x="8"/>
-        <item x="2"/>
-        <item x="10"/>
-        <item x="6"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="12"/>
-        <item x="4"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="1"/>
-        <item x="0"/>
-        <item m="1" x="4"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="15">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="13"/>
-  </colFields>
-  <colItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <pageFields count="2">
-    <pageField fld="3" hier="-1"/>
-    <pageField fld="4" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Cuenta de Estado inicio" fld="13" subtotal="count" baseField="6" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="9">
-    <chartFormat chart="5" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="5" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="9" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="10" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="11" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="12" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{28E38F05-C705-4B63-8427-947953AE6907}" name="TablaDinámica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="35">
-  <location ref="W107:Y122" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="32">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="18">
-        <item x="0"/>
-        <item x="1"/>
-        <item h="1" x="15"/>
-        <item x="2"/>
-        <item h="1" m="1" x="16"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="16">
-        <item x="1"/>
-        <item x="9"/>
-        <item x="8"/>
-        <item x="2"/>
-        <item x="10"/>
-        <item x="6"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="12"/>
-        <item x="4"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="6">
-        <item h="1" x="2"/>
-        <item h="1" x="1"/>
-        <item x="0"/>
-        <item h="1" m="1" x="4"/>
-        <item h="1" x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="13"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <pageFields count="2">
-    <pageField fld="3" hier="-1"/>
-    <pageField fld="4" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Cuenta de Estado inicio" fld="13" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="10">
-    <format dxfId="15">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="14">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="13">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="6" count="13">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-            <x v="4"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="12">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="11">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="10">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="9">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="8">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="6" count="13">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-            <x v="4"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="7">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="6">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="4">
-    <chartFormat chart="34" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="34" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="34" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="34" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6EF99BAB-2468-4B54-BA40-E9C7DB4614DE}" name="TablaDinámica3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="20">
-  <location ref="A107:D123" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="32">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="18">
-        <item x="0"/>
-        <item x="1"/>
-        <item h="1" x="15"/>
-        <item x="2"/>
-        <item h="1" m="1" x="16"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="16">
-        <item x="1"/>
-        <item x="9"/>
-        <item x="8"/>
-        <item x="2"/>
-        <item x="10"/>
-        <item x="6"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="12"/>
-        <item x="4"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="15">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="8"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <pageFields count="2">
-    <pageField fld="3" hier="-1"/>
-    <pageField fld="4" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Suma de Kilómetros" fld="19" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="6">
-    <chartFormat chart="16" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="16" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="16" format="2">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="19" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="19" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="19" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="6" count="1" selected="0">
-            <x v="12"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{238AB259-E577-48AC-B3A0-09F752F5685D}" name="TablaDinámica6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
   <location ref="A169:B185" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="43">
@@ -40772,7 +40112,7 @@
     <dataField name="Suma de Sumatoria de tiempo total sin recorrido" fld="38" baseField="6" baseItem="0" numFmtId="21"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="16">
+    <format dxfId="6">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -40799,308 +40139,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4B44BF58-179E-4C57-BD89-E6E3367D37B9}" name="TablaDinámica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34">
-  <location ref="K107:M122" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="32">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="18">
-        <item x="0"/>
-        <item x="1"/>
-        <item h="1" x="15"/>
-        <item x="2"/>
-        <item h="1" m="1" x="16"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="16">
-        <item x="1"/>
-        <item x="9"/>
-        <item x="8"/>
-        <item x="2"/>
-        <item x="10"/>
-        <item x="6"/>
-        <item x="0"/>
-        <item x="11"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="12"/>
-        <item x="4"/>
-        <item x="13"/>
-        <item x="7"/>
-        <item x="14"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="6">
-        <item h="1" x="0"/>
-        <item h="1" m="1" x="4"/>
-        <item x="1"/>
-        <item h="1" x="2"/>
-        <item h="1" x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="17"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <pageFields count="2">
-    <pageField fld="3" hier="-1"/>
-    <pageField fld="4" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Cuenta de Estado fin" fld="17" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="12">
-    <format dxfId="28">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="27">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="26">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="6" count="13">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-            <x v="4"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="25">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="24">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="17" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="23">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="22">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-    <format dxfId="21">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="20">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="6" count="13">
-            <x v="0"/>
-            <x v="1"/>
-            <x v="2"/>
-            <x v="3"/>
-            <x v="4"/>
-            <x v="5"/>
-            <x v="6"/>
-            <x v="7"/>
-            <x v="8"/>
-            <x v="9"/>
-            <x v="10"/>
-            <x v="11"/>
-            <x v="13"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="19">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="18">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="17" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="17">
-      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="4">
-    <chartFormat chart="28" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="17" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="28" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="17" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="28" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="17" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="28" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="17" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{47E67C1C-2F15-4D2B-A97A-A1B46B6F5B69}" name="TablaDinámica2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="28">
   <location ref="A57:E73" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="32">
@@ -41376,7 +40415,883 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2D330A9A-54B8-43DD-8D11-CC5633B99CDA}" name="TablaDinámica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+  <location ref="A6:E22" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="32">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="18">
+        <item x="0"/>
+        <item x="1"/>
+        <item h="1" x="15"/>
+        <item x="2"/>
+        <item h="1" m="1" x="16"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="16">
+        <item x="1"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="2"/>
+        <item x="10"/>
+        <item x="6"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="12"/>
+        <item x="4"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item m="1" x="4"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="15">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="13"/>
+  </colFields>
+  <colItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="3" hier="-1"/>
+    <pageField fld="4" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Cuenta de Estado inicio" fld="13" subtotal="count" baseField="6" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="9">
+    <chartFormat chart="5" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="5" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="9" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="10" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="11" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="12" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4B44BF58-179E-4C57-BD89-E6E3367D37B9}" name="TablaDinámica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34">
+  <location ref="K107:M122" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="32">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="18">
+        <item x="0"/>
+        <item x="1"/>
+        <item h="1" x="15"/>
+        <item x="2"/>
+        <item h="1" m="1" x="16"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="16">
+        <item x="1"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="2"/>
+        <item x="10"/>
+        <item x="6"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="12"/>
+        <item x="4"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="6">
+        <item h="1" x="0"/>
+        <item h="1" m="1" x="4"/>
+        <item x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="17"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="3" hier="-1"/>
+    <pageField fld="4" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Cuenta de Estado fin" fld="17" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="12">
+    <format dxfId="18">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="6" count="13">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="15">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="17" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="13">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="12">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="11">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="6" count="13">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="9">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="17" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="7">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="4">
+    <chartFormat chart="28" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="17" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="28" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="17" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="28" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="17" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="28" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="17" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{28E38F05-C705-4B63-8427-947953AE6907}" name="TablaDinámica5" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="35">
+  <location ref="W107:Y122" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="32">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="18">
+        <item x="0"/>
+        <item x="1"/>
+        <item h="1" x="15"/>
+        <item x="2"/>
+        <item h="1" m="1" x="16"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="16">
+        <item x="1"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="2"/>
+        <item x="10"/>
+        <item x="6"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="12"/>
+        <item x="4"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="6">
+        <item h="1" x="2"/>
+        <item h="1" x="1"/>
+        <item x="0"/>
+        <item h="1" m="1" x="4"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="13"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="3" hier="-1"/>
+    <pageField fld="4" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Cuenta de Estado inicio" fld="13" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="10">
+    <format dxfId="28">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="27">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="26">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="6" count="13">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="24">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="23">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="22">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="21">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="6" count="13">
+            <x v="0"/>
+            <x v="1"/>
+            <x v="2"/>
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+            <x v="8"/>
+            <x v="9"/>
+            <x v="10"/>
+            <x v="11"/>
+            <x v="13"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="20">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="19">
+      <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="4">
+    <chartFormat chart="34" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="34" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="34" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="34" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E0966AFF-8B15-4A0E-BE48-1F64EB76CB37}" name="TablaDinámica7" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="57">
   <location ref="AI107:AJ122" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="32">
@@ -41620,6 +41535,259 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6EF99BAB-2468-4B54-BA40-E9C7DB4614DE}" name="TablaDinámica3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="20">
+  <location ref="A107:D123" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="32">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="18">
+        <item x="0"/>
+        <item x="1"/>
+        <item h="1" x="15"/>
+        <item x="2"/>
+        <item h="1" m="1" x="16"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="16">
+        <item x="1"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="2"/>
+        <item x="10"/>
+        <item x="6"/>
+        <item x="0"/>
+        <item x="11"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="12"/>
+        <item x="4"/>
+        <item x="13"/>
+        <item x="7"/>
+        <item x="14"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="15">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="8"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="3" hier="-1"/>
+    <pageField fld="4" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Suma de Kilómetros" fld="19" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="16" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="16" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="16" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="19" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="19" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="19" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="6" count="1" selected="0">
+            <x v="12"/>
+          </reference>
+          <reference field="8" count="1" selected="0">
+            <x v="1"/>
           </reference>
         </references>
       </pivotArea>
@@ -66699,54 +66867,854 @@
       <c r="AN191" s="9"/>
     </row>
     <row r="192" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A192" s="9" t="s">
+        <v>1671</v>
+      </c>
+      <c r="B192" s="9" t="s">
+        <v>1672</v>
+      </c>
+      <c r="C192" s="9" t="s">
+        <v>1673</v>
+      </c>
+      <c r="D192" s="9" t="s">
+        <v>1600</v>
+      </c>
+      <c r="E192" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F192" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G192" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H192" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I192" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J192" s="9">
+        <v>2110</v>
+      </c>
+      <c r="K192" s="9" t="s">
+        <v>1674</v>
+      </c>
+      <c r="L192" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M192" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="N192" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="O192" s="9" t="s">
+        <v>1675</v>
+      </c>
+      <c r="P192" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q192" s="10">
+        <v>3.6168981481481483E-2</v>
+      </c>
+      <c r="R192" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="S192" s="10">
+        <v>0.20383101851851851</v>
+      </c>
+      <c r="T192" s="9">
+        <v>26.300999999999998</v>
+      </c>
+      <c r="U192" s="9">
+        <v>7.48</v>
+      </c>
+      <c r="V192" s="10">
+        <v>0.14656250000000001</v>
+      </c>
+      <c r="W192" s="10">
+        <v>7.8009259259259264E-2</v>
+      </c>
+      <c r="X192" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y192" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z192" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA192" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB192" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC192" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD192" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE192" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF192" s="9" t="s">
+        <v>1676</v>
+      </c>
+      <c r="AG192" s="9" t="s">
+        <v>1677</v>
+      </c>
+      <c r="AH192" s="9">
+        <v>6.2701349999999998</v>
+      </c>
+      <c r="AI192" s="9">
+        <v>-75.601358000000005</v>
+      </c>
+      <c r="AJ192" s="9" t="s">
+        <v>1678</v>
+      </c>
+      <c r="AK192" s="9">
+        <v>6.2463579999999999</v>
+      </c>
+      <c r="AL192" s="9">
+        <v>-75.604612000000003</v>
+      </c>
       <c r="AN192" s="9"/>
     </row>
-    <row r="193" spans="40:40" x14ac:dyDescent="0.25">
-      <c r="AN193" s="9"/>
+    <row r="193" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A193" s="9" t="s">
+        <v>1679</v>
+      </c>
+      <c r="B193" s="9" t="s">
+        <v>1680</v>
+      </c>
+      <c r="C193" s="9" t="s">
+        <v>1681</v>
+      </c>
+      <c r="D193" s="9" t="s">
+        <v>1600</v>
+      </c>
+      <c r="E193" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F193" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G193" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H193" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I193" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J193" s="9">
+        <v>3418</v>
+      </c>
+      <c r="K193" s="9" t="s">
+        <v>1682</v>
+      </c>
+      <c r="L193" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M193" s="10">
+        <v>0.18044956018518521</v>
+      </c>
+      <c r="N193" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="O193" s="9" t="s">
+        <v>1683</v>
+      </c>
+      <c r="P193" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q193" s="10">
+        <v>9.5990509259259258E-3</v>
+      </c>
+      <c r="R193" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="S193" s="10">
+        <v>7.9149490740740736E-2</v>
+      </c>
+      <c r="T193" s="9">
+        <v>16.713999999999999</v>
+      </c>
+      <c r="U193" s="9">
+        <v>19.91</v>
+      </c>
+      <c r="V193" s="10">
+        <v>3.4982083333333337E-2</v>
+      </c>
+      <c r="W193" s="10">
+        <v>2.1908865740740739E-2</v>
+      </c>
+      <c r="X193" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y193" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z193" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA193" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB193" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC193" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD193" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE193" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF193" s="9" t="s">
+        <v>1684</v>
+      </c>
+      <c r="AG193" s="9" t="s">
+        <v>1685</v>
+      </c>
+      <c r="AH193" s="9">
+        <v>6.2513550000000002</v>
+      </c>
+      <c r="AI193" s="9">
+        <v>-75.607427999999999</v>
+      </c>
+      <c r="AJ193" s="9" t="s">
+        <v>1686</v>
+      </c>
+      <c r="AK193" s="9">
+        <v>6.2725660000000003</v>
+      </c>
+      <c r="AL193" s="9">
+        <v>-75.602164000000002</v>
+      </c>
+      <c r="AN193" s="9" t="s">
+        <v>1726</v>
+      </c>
     </row>
-    <row r="194" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A194" s="9" t="s">
+        <v>1687</v>
+      </c>
+      <c r="B194" s="9" t="s">
+        <v>1688</v>
+      </c>
+      <c r="C194" s="9" t="s">
+        <v>1689</v>
+      </c>
+      <c r="D194" s="9" t="s">
+        <v>1600</v>
+      </c>
+      <c r="E194" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F194" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G194" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="H194" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="I194" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J194" s="9">
+        <v>1869</v>
+      </c>
+      <c r="K194" s="9" t="s">
+        <v>1690</v>
+      </c>
+      <c r="L194" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M194" s="10">
+        <v>1.8518518518518519E-3</v>
+      </c>
+      <c r="N194" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="O194" s="9" t="s">
+        <v>1691</v>
+      </c>
+      <c r="P194" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q194" s="10">
+        <v>1.0706018518518519E-2</v>
+      </c>
+      <c r="R194" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="S194" s="10">
+        <v>0.2374421296296296</v>
+      </c>
+      <c r="T194" s="9">
+        <v>34.732999999999997</v>
+      </c>
+      <c r="U194" s="9">
+        <v>19.53</v>
+      </c>
+      <c r="V194" s="10">
+        <v>7.4097222222222217E-2</v>
+      </c>
+      <c r="W194" s="10">
+        <v>3.2002314814814817E-2</v>
+      </c>
+      <c r="X194" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y194" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z194" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA194" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB194" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC194" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD194" s="9">
+        <v>3</v>
+      </c>
+      <c r="AE194" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF194" s="9" t="s">
+        <v>1692</v>
+      </c>
+      <c r="AG194" s="9" t="s">
+        <v>1693</v>
+      </c>
+      <c r="AH194" s="9">
+        <v>6.2719529999999999</v>
+      </c>
+      <c r="AI194" s="9">
+        <v>-75.540672999999998</v>
+      </c>
+      <c r="AJ194" s="9" t="s">
+        <v>1694</v>
+      </c>
+      <c r="AK194" s="9">
+        <v>6.2644299999999999</v>
+      </c>
+      <c r="AL194" s="9">
+        <v>-75.570660000000004</v>
+      </c>
       <c r="AN194" s="9"/>
     </row>
-    <row r="195" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A195" s="9" t="s">
+        <v>1695</v>
+      </c>
+      <c r="B195" s="9" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C195" s="9" t="s">
+        <v>1697</v>
+      </c>
+      <c r="D195" s="9" t="s">
+        <v>1600</v>
+      </c>
+      <c r="E195" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F195" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G195" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="H195" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="I195" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J195" s="9">
+        <v>7141</v>
+      </c>
+      <c r="K195" s="9" t="s">
+        <v>1698</v>
+      </c>
+      <c r="L195" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M195" s="10">
+        <v>1.9467592592592588E-2</v>
+      </c>
+      <c r="N195" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="O195" s="9" t="s">
+        <v>1699</v>
+      </c>
+      <c r="P195" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q195" s="10">
+        <v>1.5127314814814821E-2</v>
+      </c>
+      <c r="R195" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="S195" s="10">
+        <v>0.28459490740740739</v>
+      </c>
+      <c r="T195" s="9">
+        <v>95.653000000000006</v>
+      </c>
+      <c r="U195" s="9">
+        <v>18.7</v>
+      </c>
+      <c r="V195" s="10">
+        <v>0.21315972222222221</v>
+      </c>
+      <c r="W195" s="10">
+        <v>4.5879629629629631E-2</v>
+      </c>
+      <c r="X195" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y195" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE195" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="AF195" s="9" t="s">
+        <v>1700</v>
+      </c>
+      <c r="AG195" s="9" t="s">
+        <v>1701</v>
+      </c>
+      <c r="AH195" s="9">
+        <v>6.2903630000000001</v>
+      </c>
+      <c r="AI195" s="9">
+        <v>-75.546538999999996</v>
+      </c>
+      <c r="AJ195" s="9" t="s">
+        <v>1702</v>
+      </c>
+      <c r="AK195" s="9">
+        <v>6.2903770000000003</v>
+      </c>
+      <c r="AL195" s="9">
+        <v>-75.546586000000005</v>
+      </c>
       <c r="AN195" s="9"/>
     </row>
-    <row r="196" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A196" s="9" t="s">
+        <v>1703</v>
+      </c>
+      <c r="B196" s="9" t="s">
+        <v>1704</v>
+      </c>
+      <c r="C196" s="9" t="s">
+        <v>1705</v>
+      </c>
+      <c r="D196" s="9" t="s">
+        <v>1600</v>
+      </c>
+      <c r="E196" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F196" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G196" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H196" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="I196" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J196" s="9">
+        <v>1651</v>
+      </c>
+      <c r="K196" s="9" t="s">
+        <v>1706</v>
+      </c>
+      <c r="L196" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M196" s="10">
+        <v>1.1458333333333329E-3</v>
+      </c>
+      <c r="N196" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="O196" s="9" t="s">
+        <v>1707</v>
+      </c>
+      <c r="P196" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q196" s="10">
+        <v>6.9444444444444447E-4</v>
+      </c>
+      <c r="R196" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="S196" s="10">
+        <v>0.2504513888888889</v>
+      </c>
+      <c r="T196" s="9">
+        <v>19.93</v>
+      </c>
+      <c r="U196" s="9">
+        <v>3.93</v>
+      </c>
+      <c r="V196" s="10">
+        <v>0.21122685185185189</v>
+      </c>
+      <c r="W196" s="10">
+        <v>0.1576967592592593</v>
+      </c>
+      <c r="X196" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y196" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z196" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA196" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB196" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC196" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD196" s="9">
+        <v>1</v>
+      </c>
+      <c r="AE196" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="AF196" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="AG196" s="9" t="s">
+        <v>1708</v>
+      </c>
+      <c r="AH196" s="9">
+        <v>6.2524670000000002</v>
+      </c>
+      <c r="AI196" s="9">
+        <v>-75.551827000000003</v>
+      </c>
+      <c r="AJ196" s="9" t="s">
+        <v>1709</v>
+      </c>
+      <c r="AK196" s="9">
+        <v>6.2518120000000001</v>
+      </c>
+      <c r="AL196" s="9">
+        <v>-75.551810000000003</v>
+      </c>
       <c r="AN196" s="9"/>
     </row>
-    <row r="197" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A197" s="9" t="s">
+        <v>1710</v>
+      </c>
+      <c r="B197" s="9" t="s">
+        <v>1711</v>
+      </c>
+      <c r="C197" s="9" t="s">
+        <v>1712</v>
+      </c>
+      <c r="D197" s="9" t="s">
+        <v>1600</v>
+      </c>
+      <c r="E197" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F197" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="G197" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="H197" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="I197" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J197" s="9">
+        <v>11062</v>
+      </c>
+      <c r="K197" s="9" t="s">
+        <v>1713</v>
+      </c>
+      <c r="L197" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M197" s="10">
+        <v>2.2600856481481479E-2</v>
+      </c>
+      <c r="N197" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="O197" s="9" t="s">
+        <v>1714</v>
+      </c>
+      <c r="P197" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q197" s="10">
+        <v>5.5555555555555556E-4</v>
+      </c>
+      <c r="R197" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="S197" s="10">
+        <v>0.27315641203703711</v>
+      </c>
+      <c r="T197" s="9">
+        <v>54.726999999999997</v>
+      </c>
+      <c r="U197" s="9">
+        <v>12.98</v>
+      </c>
+      <c r="V197" s="10">
+        <v>0.17561365740740739</v>
+      </c>
+      <c r="W197" s="10">
+        <v>0.1248032407407407</v>
+      </c>
+      <c r="X197" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y197" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z197" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA197" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB197" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC197" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD197" s="9">
+        <v>2</v>
+      </c>
+      <c r="AE197" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="AF197" s="9" t="s">
+        <v>1715</v>
+      </c>
+      <c r="AG197" s="9" t="s">
+        <v>1716</v>
+      </c>
+      <c r="AH197" s="9">
+        <v>6.2689079999999997</v>
+      </c>
+      <c r="AI197" s="9">
+        <v>-75.598983000000004</v>
+      </c>
+      <c r="AJ197" s="9" t="s">
+        <v>1717</v>
+      </c>
+      <c r="AK197" s="9">
+        <v>6.2397520000000002</v>
+      </c>
+      <c r="AL197" s="9">
+        <v>-75.575770000000006</v>
+      </c>
       <c r="AN197" s="9"/>
     </row>
-    <row r="198" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A198" s="9" t="s">
+        <v>1718</v>
+      </c>
+      <c r="B198" s="9" t="s">
+        <v>1719</v>
+      </c>
+      <c r="C198" s="9" t="s">
+        <v>1720</v>
+      </c>
+      <c r="D198" s="9" t="s">
+        <v>1664</v>
+      </c>
+      <c r="E198" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F198" s="9" t="s">
+        <v>455</v>
+      </c>
+      <c r="G198" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H198" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I198" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="J198" s="9">
+        <v>1907</v>
+      </c>
+      <c r="K198" s="9" t="s">
+        <v>1721</v>
+      </c>
+      <c r="L198" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="M198" s="10">
+        <v>1.621527777777778E-2</v>
+      </c>
+      <c r="N198" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="O198" s="9" t="s">
+        <v>1722</v>
+      </c>
+      <c r="P198" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q198" s="10">
+        <v>3.668981481481481E-3</v>
+      </c>
+      <c r="R198" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="S198" s="10">
+        <v>0.23745370370370369</v>
+      </c>
+      <c r="T198" s="9">
+        <v>25.712</v>
+      </c>
+      <c r="U198" s="9">
+        <v>7.32</v>
+      </c>
+      <c r="V198" s="10">
+        <v>0.1464236111111111</v>
+      </c>
+      <c r="W198" s="10">
+        <v>0.1012268518518518</v>
+      </c>
+      <c r="X198" s="10">
+        <v>0</v>
+      </c>
+      <c r="Y198" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z198" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA198" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB198" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC198" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD198" s="9">
+        <v>0</v>
+      </c>
+      <c r="AE198" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF198" s="9" t="s">
+        <v>1723</v>
+      </c>
+      <c r="AG198" s="9" t="s">
+        <v>1724</v>
+      </c>
+      <c r="AH198" s="9">
+        <v>6.2477510000000001</v>
+      </c>
+      <c r="AI198" s="9">
+        <v>-75.614997000000002</v>
+      </c>
+      <c r="AJ198" s="9" t="s">
+        <v>1725</v>
+      </c>
+      <c r="AK198" s="9">
+        <v>6.2476419999999999</v>
+      </c>
+      <c r="AL198" s="9">
+        <v>-75.614914999999996</v>
+      </c>
       <c r="AN198" s="9"/>
     </row>
-    <row r="199" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN199" s="9"/>
     </row>
-    <row r="200" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN200" s="9"/>
     </row>
-    <row r="201" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN201" s="9"/>
     </row>
-    <row r="202" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN202" s="9"/>
     </row>
-    <row r="203" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN203" s="9"/>
     </row>
-    <row r="204" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN204" s="9"/>
     </row>
-    <row r="205" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN205" s="9"/>
     </row>
-    <row r="206" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN206" s="9"/>
     </row>
-    <row r="207" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN207" s="9"/>
     </row>
-    <row r="208" spans="40:40" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:40" x14ac:dyDescent="0.25">
       <c r="AN208" s="9"/>
     </row>
     <row r="209" spans="40:40" x14ac:dyDescent="0.25">

</xml_diff>